<commit_message>
Malvinas: se saca de la plantilla la firma y el sello del capitan de BELTOKYO
La plantilla traia una imagen con la firma y el sello de otro buque; salia en todos los documentos.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/docgen/templates/malvinas.xlsx
+++ b/app/docgen/templates/malvinas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\lineup\app\docgen\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BEB6275-449D-4A84-90E9-99B0841C66B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF62463B-8291-4804-8F22-B2F260D304B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-6465" windowWidth="24240" windowHeight="13020" xr2:uid="{775E3EBF-A09A-4259-B1F2-E133807AE976}"/>
   </bookViews>
@@ -347,85 +347,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>144780</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>53340</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>548640</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4EB460B4-6A20-4737-995B-3CAB93D58FA8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="3162300" y="8420100"/>
-          <a:ext cx="2748915" cy="1062990"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1535,6 +1456,5 @@
   <pageMargins left="0.17" right="0.16" top="0.23" bottom="0.2" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="96" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Malvinas: plantilla desde el formulario limpio del usuario (sin firma ni sello)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/docgen/templates/malvinas.xlsx
+++ b/app/docgen/templates/malvinas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\lineup\app\docgen\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF62463B-8291-4804-8F22-B2F260D304B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{67C0188B-DDA2-439E-959E-6285727D2302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-6465" windowWidth="24240" windowHeight="13020" xr2:uid="{775E3EBF-A09A-4259-B1F2-E133807AE976}"/>
   </bookViews>
@@ -294,6 +294,33 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -301,33 +328,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1154,64 +1154,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="3" spans="1:12" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
     </row>
     <row r="5" spans="1:12" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
       <c r="J9"/>
       <c r="K9" s="2"/>
       <c r="L9"/>
@@ -1222,71 +1222,71 @@
       <c r="L10" s="3"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
       <c r="E20" s="6" t="s">
         <v>11</v>
       </c>
@@ -1295,11 +1295,11 @@
       <c r="A22" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="21">
+      <c r="C22" s="19">
         <f>C20</f>
         <v>0</v>
       </c>
-      <c r="D22" s="15"/>
+      <c r="D22" s="20"/>
       <c r="E22" s="7" t="s">
         <v>13</v>
       </c>
@@ -1308,9 +1308,9 @@
       <c r="A24" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
       <c r="G24" s="6" t="s">
         <v>15</v>
       </c>
@@ -1336,32 +1336,32 @@
       <c r="A28" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
       <c r="D28" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F28" s="6"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="23">
         <f>B28</f>
         <v>0</v>
       </c>
-      <c r="C30" s="14"/>
+      <c r="C30" s="23"/>
       <c r="D30" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G30" s="15">
+      <c r="G30" s="20">
         <f>G28</f>
         <v>0</v>
       </c>
-      <c r="H30" s="15"/>
+      <c r="H30" s="20"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
@@ -1434,12 +1434,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A9:H9"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A14:H14"/>
@@ -1452,6 +1446,12 @@
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="G30:H30"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A9:H9"/>
   </mergeCells>
   <pageMargins left="0.17" right="0.16" top="0.23" bottom="0.2" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="96" orientation="portrait" r:id="rId1"/>

</xml_diff>